<commit_message>
docs: GK-105 leva para o Drive o preenchimento das planilhas com a situação de 27/10
US: GK-105 [US-105] Planilhas da disciplina: DoD, Plano de Qualidade e Análise de Riscos
Planilhas de origem: GK-38 (DoD), GK-36 (Plano de Qualidade) e GK-64 (Análise de Riscos)

O preenchimento de 26/10 ficou só no repositório; o Drive seguia na versão
anterior. As planilhas partem agora da versão do Drive e trazem a situação
de 27/10, com o login (GK-8, PR #10) já no main: na Análise de Riscos, a
situação dos quatro riscos que mudaram; no Plano de Qualidade, o resultado
R1 dos 15 itens (rota protegida testada, 29 de 29 execuções do CI verdes,
0 de 10 PRs com revisão, 18 de 28 pontos); na DoD, Sprint 1 com planilha
de riscos atualizada e testes de segurança passando. Estas são as versões
enviadas ao Drive em Gerenciar versões, mantendo os links do README.
</commit_message>
<xml_diff>
--- a/docs/Analise-de-Riscos-Baseada-em-Defeitos.xlsx
+++ b/docs/Analise-de-Riscos-Baseada-em-Defeitos.xlsx
@@ -1622,7 +1622,7 @@
       <c r="J8" s="20" t="inlineStr">
         <is>
           <t>Hash bcrypt no cadastro e teste que garante que a senha não aparece no banco nem na resposta. Issue GK-43 (Release 1, Sprint 1). Responsável: Pedro
-Situação em 26/10/2026: atendido no main: restrição bcrypt em core.usuarios (GK-90), hash no cadastro (GK-7, PR #9) e testes do driver DA-SEG-I1-01 (GK-69, PR #6) no CI verde.</t>
+Situação em 27/10/2026: atendido no main: restrição bcrypt em core.usuarios (GK-90), hash no cadastro (GK-7, PR #9) e testes do driver DA-SEG-I1-01 (GK-69, PR #6) no CI verde.</t>
         </is>
       </c>
       <c r="K8" s="20">
@@ -1737,7 +1737,7 @@
       <c r="J10" s="20" t="inlineStr">
         <is>
           <t>Uma única verificação de autenticação que valida expiração e perfil, com teste para cada rota protegida. Issues GK-44 (Release 1, Sprint 1) e GK-50 (Release 3). Responsável: Rodrigo
-Situação em 26/10/2026: em andamento: login e sessão no PR #10 (GK-8), ainda fora do main; testes de token vencido, adulterado e com perfil errado a conferir.</t>
+Situação em 27/10/2026: parcial: login e sessão no main (GK-8, PR #10) com uma única verificação do token, que confere a expiração e se o usuário segue ativo; testes de token ausente, inválido e expirado no CI verde. Falta o teste de perfil errado, que depende das rotas de administrador (GK-50, Release 3).</t>
         </is>
       </c>
       <c r="K10" s="20">
@@ -1915,7 +1915,7 @@
       <c r="J16" s="20" t="inlineStr">
         <is>
           <t>Reservar a chave dentro de uma transação com bloqueio de linha (SELECT ... FOR UPDATE SKIP LOCKED) e manter o teste de concorrência no CI. Issues GK-46 e GK-15 (Release 2, Sprints 2 e 3). Responsável: Pedro
-Situação em 26/10/2026: modelo previsto no DER v1.0 (GK-103/GK-104): chave_id único em vendas.itens_pedido; implementação e teste de concorrência na Release 2.</t>
+Situação em 27/10/2026: modelo previsto no DER v1.0 (GK-103/GK-104): chave_id único em vendas.itens_pedido; implementação e teste de concorrência na Release 2.</t>
         </is>
       </c>
       <c r="K16" s="20">
@@ -2209,7 +2209,7 @@
       <c r="J25" s="20" t="inlineStr">
         <is>
           <t>Formato único de erro na API com mensagem em português e exibição ao lado do campo no front. Issue GK-45 (Release 1, Sprint 1). Responsável: Wagner
-Situação em 26/10/2026: parcial: o cadastro (GK-7) responde em português para e-mail repetido e senha curta e não expõe detalhes técnicos; falta o login e o checklist do QA.</t>
+Situação em 27/10/2026: parcial: cadastro (GK-7) e login (GK-8) respondem em português (e-mail repetido, senha curta, e-mail ou senha incorretos) sem expor detalhes técnicos; falta a mensagem ao lado do campo no front e o checklist do QA.</t>
         </is>
       </c>
       <c r="K25" s="20">

</xml_diff>

<commit_message>
docs: GK-105 fecha as planilhas com o pré-encerramento da Sprint 1
US: GK-105 [US-105] Planilhas da disciplina: DoD, Plano de Qualidade e Análise de Riscos

Atualiza as três planilhas com o que foi registrado no Jira em 28/10/2026:
8 de 9 US concluídas (27 de 28 pontos), GK-106 concluído, QA do Wagner
e aceite do PO comunicados ao SM, CI da main 32/32 e os 3 drivers da
Release 1 concluídos. A falta de review nos 13 PRs fica como "Não" na
DoD da Sprint, com o plano da Q-11.
</commit_message>
<xml_diff>
--- a/docs/Analise-de-Riscos-Baseada-em-Defeitos.xlsx
+++ b/docs/Analise-de-Riscos-Baseada-em-Defeitos.xlsx
@@ -1596,7 +1596,7 @@
       <c r="J8" s="20" t="inlineStr">
         <is>
           <t>Hash bcrypt no cadastro e teste que garante que a senha não aparece no banco nem na resposta. Issue GK-43 (Release 1, Sprint 1). Responsável: Pedro
-Situação em 28/10/2026: atendido tecnicamente no main: restrição bcrypt em core.usuarios (GK-90), cadastro GK-7/PR #9 e driver GK-69/PR #6. Regressão local: 87/87 testes backend, 27/27 E2E e 9/9 integrações; CI da main 31/31 verde. Validação formal do QA permanece pendente.</t>
+Situação em 28/10/2026: atendido no main: restrição bcrypt em core.usuarios (GK-90), cadastro GK-7/PR #9 e driver GK-69 Concluído. Regressão: 87/87 backend, 27/27 E2E e 9/9 integrações; CI da main 32/32 verde. QA de Wagner confirmado, registrado pelo SM na GK-80.</t>
         </is>
       </c>
       <c r="K8" s="20">
@@ -1711,7 +1711,7 @@
       <c r="J10" s="20" t="inlineStr">
         <is>
           <t>Uma única verificação de autenticação que valida expiração e perfil, com teste para cada rota protegida. Issues GK-44 (Release 1, Sprint 1) e GK-50 (Release 3). Responsável: Rodrigo
-Situação em 27/10/2026: parcial: login e sessão no main (GK-8, PR #10), com validação de expiração e usuário ativo; token ausente, inválido e expirado cobertos na regressão automatizada. Falta o teste de perfil errado, dependente das rotas de administrador (GK-50, Release 3), e a validação formal do QA.</t>
+Situação em 28/10/2026: parcial: login e sessão no main (GK-8, PR #10) e driver GK-71 Concluído; token ausente, inválido e expirado cobertos na regressão, com QA confirmado (GK-83). Falta o teste de perfil errado, que depende das rotas de administrador (GK-50, Release 3).</t>
         </is>
       </c>
       <c r="K10" s="20">
@@ -2183,7 +2183,7 @@
       <c r="J25" s="20" t="inlineStr">
         <is>
           <t>Formato único de erro na API com mensagem em português e exibição ao lado do campo no front. Issue GK-45 (Release 1, Sprint 1). Responsável: Wagner
-Situação em 27/10/2026: parcial: cadastro e login respondem em português sem expor detalhes técnicos; regressão local com 27/27 cenários E2E e 9/9 integrações aprovada. Falta confirmar a exibição junto ao campo e registrar o checklist formal do QA.</t>
+Situação em 28/10/2026: atendido na Release 1: cadastro e login respondem em português sem expor detalhes técnicos (GK-45 e driver GK-76 Concluídos); 27/27 cenários E2E e 9/9 integrações. QA confirmado pelo SM; checklist individual do QA não anexado.</t>
         </is>
       </c>
       <c r="K25" s="20">

</xml_diff>